<commit_message>
Stamp the audit commit in the revision history; state exactly what the rebuild test covered
The dated revision history now names commit 1b845d0 and its time for each audit entry
(data/extension_staging/commit_stamp_audit.json). REBUILD.md and the response to finding F21
say what was tested: steps 1-11 in a fresh clone reproduced every tracked file, the two
.xlsx files cell for cell; the Chrome render of the PDF extracts, the link sweep and the
network collectors were not repeated there.

The checksum manifest treated .gitignore and .gitattributes as binary, so their recorded
hashes were of the CRLF working copies rather than of the bytes git stores; scripts/served.py
now treats them as text and 78_verify_checksums.py matches all 1,353 rows. The Data page
quotes the size of the final manifest.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -67075,6 +67075,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>value corrected</t>
@@ -67137,6 +67147,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>value corrected</t>
@@ -67199,6 +67219,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>value corrected</t>
@@ -67261,6 +67291,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>value corrected</t>
@@ -67323,6 +67363,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>value corrected</t>
@@ -67385,6 +67435,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>value deleted</t>
@@ -67447,6 +67507,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>source re-cited</t>
@@ -67509,6 +67579,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>values added</t>
@@ -67571,6 +67651,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>grade changed</t>
@@ -67633,6 +67723,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>flag changed</t>
@@ -67695,6 +67795,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>value reclassified</t>
@@ -67757,6 +67867,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>evidence added</t>
@@ -67802,6 +67922,16 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1b845d0</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">

</xml_diff>

<commit_message>
Stamp the re-audit commit in the revision history
The dated revision history now names commit f093c3e and its time for the re-audit entries
(data/extension_staging/commit_stamp_reaudit.json).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -68029,6 +68029,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>21:18</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>f093c3e</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>flagged as derived</t>
@@ -68091,6 +68101,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>21:18</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>f093c3e</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>flag changed</t>
@@ -68153,6 +68173,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>21:18</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>f093c3e</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>re-verified</t>
@@ -68203,6 +68233,16 @@
       <c r="A31" t="inlineStr">
         <is>
           <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>21:18</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>f093c3e</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">

</xml_diff>

<commit_message>
Stamp the health-expenditure commit in the revision history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -75547,6 +75547,16 @@
           <t>2026-10-17</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>d05a8d6</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>variable added</t>
@@ -75607,6 +75617,16 @@
       <c r="A34" t="inlineStr">
         <is>
           <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>d05a8d6</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">

</xml_diff>

<commit_message>
Stamp the 2026-10-18 commit in the revision history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -75791,6 +75791,16 @@
           <t>2026-10-18</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>cedba02</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>note amended</t>
@@ -75853,6 +75863,16 @@
           <t>2026-10-18</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>cedba02</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>documentation corrected</t>
@@ -75905,6 +75925,16 @@
           <t>2026-10-18</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>cedba02</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>values added</t>
@@ -75967,6 +75997,16 @@
           <t>2026-10-18</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>cedba02</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>documentation corrected</t>
@@ -76017,6 +76057,16 @@
       <c r="A39" t="inlineStr">
         <is>
           <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>cedba02</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">

</xml_diff>

<commit_message>
Stamp the 2026-10-21 commit in the revision history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -83589,6 +83589,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>4b161c9</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>variable added</t>
@@ -83651,6 +83661,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>4b161c9</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>documentation corrected</t>
@@ -83701,6 +83721,16 @@
       <c r="A42" t="inlineStr">
         <is>
           <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>4b161c9</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">

</xml_diff>

<commit_message>
Stamp the 2026-10-26 commit in the revision history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -90929,6 +90929,16 @@
           <t>2026-10-26</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ea42395</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>variable added</t>

</xml_diff>

<commit_message>
Stamp the 2026-10-29 commit in the revision history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -97251,6 +97251,16 @@
           <t>2026-10-29</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>8fd6c7f</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>variable added</t>

</xml_diff>

<commit_message>
Stamp the 2026-10-29 correction commit in the revision history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CLEAN_country_year_panel_2010-2022.xlsx
+++ b/data/CLEAN_country_year_panel_2010-2022.xlsx
@@ -97323,6 +97323,16 @@
           <t>2026-10-29</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:48</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>bfc542f</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>documentation corrected</t>
@@ -97373,6 +97383,16 @@
       <c r="A46" t="inlineStr">
         <is>
           <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>22:48</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>bfc542f</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">

</xml_diff>